<commit_message>
chore: personalize submission form, AI_USE, and REPORT with candidate details (Tharun S)
</commit_message>
<xml_diff>
--- a/IncuBrix_Assessment_4_Distribution_Long_Tail_Destination_Network_Submission_Form.xlsx
+++ b/IncuBrix_Assessment_4_Distribution_Long_Tail_Destination_Network_Submission_Form.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>IncuBrix Placement Candidate</t>
+          <t>Tharun S</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,11 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n"/>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>tharun.suresh@outlook.com</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="19.5" customHeight="1" s="13">
       <c r="A6" s="19" t="inlineStr">
@@ -835,7 +839,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>http://localhost:8000</t>
+          <t>http://localhost:8001</t>
         </is>
       </c>
     </row>
@@ -873,7 +877,11 @@
           <t>Demo video URL (max 8 min, unedited)</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n"/>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Local reproduction available via ./run_tests.sh &amp; Web UI at http://localhost:8001</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="19.5" customHeight="1" s="13">
       <c r="A14" s="19" t="inlineStr">
@@ -2652,7 +2660,7 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>IncuBrix Placement Candidate</t>
+          <t>Tharun S</t>
         </is>
       </c>
     </row>

</xml_diff>